<commit_message>
Documentation for TEASER and OpenDHW generally ready, small bugfix of start time in example 17
</commit_message>
<xml_diff>
--- a/uesgraphs/data/uesgraphs_parameters_template_pp.xlsx
+++ b/uesgraphs/data/uesgraphs_parameters_template_pp.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="120">
   <si>
     <t xml:space="preserve">uesgraphs Parameter Template</t>
   </si>
@@ -33,7 +33,7 @@
     <t xml:space="preserve">Version: 3.0</t>
   </si>
   <si>
-    <t xml:space="preserve">This Excel template provides parameters for generating Modelica district heating/cooling network models.</t>
+    <t xml:space="preserve">This Excel template provides parameters for generating pandapipes district heating/cooling network models.</t>
   </si>
   <si>
     <t xml:space="preserve">Fill in the parameters in each sheet, then use this file with uesgraphs.create_model().</t>
@@ -162,7 +162,7 @@
     <t xml:space="preserve">dynamic</t>
   </si>
   <si>
-    <t xml:space="preserve">Mode for dynamic or static simulation must be set either to „dynamic“ or to „static“</t>
+    <t xml:space="preserve">Mode for dynamic or static simulation must be set either to „dynamic“ or to „static“ or  „transient“ for full pandapipes simulation</t>
   </si>
   <si>
     <t xml:space="preserve">save_params_to_csv</t>
@@ -189,12 +189,27 @@
     <t xml:space="preserve">Ground depth for embedded pipes</t>
   </si>
   <si>
+    <t xml:space="preserve">temp_dT_dhw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only for DHW calc, temperature difference between freshwater and average DHW outlet temperature </t>
+  </si>
+  <si>
+    <t xml:space="preserve">mean_drawoff_vol_per_day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L/day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only for DHW calc, Mean drawoff volume per person for a day</t>
+  </si>
+  <si>
     <t xml:space="preserve">dT_Network</t>
   </si>
   <si>
-    <t xml:space="preserve">K</t>
-  </si>
-  <si>
     <t xml:space="preserve">Temperature difference in network</t>
   </si>
   <si>
@@ -216,6 +231,9 @@
     <t xml:space="preserve">pIn</t>
   </si>
   <si>
+    <t xml:space="preserve">Pa</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fixed suppy pressure</t>
   </si>
   <si>
@@ -226,9 +244,6 @@
   </si>
   <si>
     <t xml:space="preserve">pReturn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pa</t>
   </si>
   <si>
     <t xml:space="preserve">Default return pressure based on pIn and dpFlow</t>
@@ -379,7 +394,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="#,##0.000"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -1186,7 +1201,7 @@
         <v>40</v>
       </c>
       <c r="B4" s="14" t="n">
-        <f aca="false">3600*24</f>
+        <f aca="false">86400</f>
         <v>86400</v>
       </c>
       <c r="C4" s="5" t="s">
@@ -1250,8 +1265,34 @@
         <v>53</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>59</v>
+      </c>
+    </row>
     <row r="11" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1298,44 +1339,44 @@
     </row>
     <row r="2" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B2" s="14" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>55</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B3" s="14" t="n">
         <v>4180</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B4" s="18" t="n">
-        <v>323.15</v>
+        <v>302.15</v>
       </c>
       <c r="C4" s="15" t="s">
         <v>55</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E4" s="15"/>
     </row>
@@ -1403,67 +1444,75 @@
     </row>
     <row r="2" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B2" s="14" t="n">
-        <v>800000</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>63</v>
-      </c>
+        <v>230000</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="E2" s="15"/>
     </row>
     <row r="3" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="B3" s="18" t="n">
-        <v>600000</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>65</v>
-      </c>
+        <v>30000</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="E3" s="15"/>
     </row>
     <row r="4" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B4" s="14" t="n">
         <f aca="false">B2-B3</f>
         <v>200000</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B5" s="14" t="n">
-        <v>353.15</v>
+        <v>319.15</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>55</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>323.15</v>
+        <v>302.15</v>
       </c>
       <c r="C6" s="15" t="s">
         <v>55</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E6" s="15"/>
     </row>
@@ -1515,44 +1564,44 @@
     </row>
     <row r="2" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B2" s="19" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B3" s="19" t="n">
-        <v>0.03</v>
+        <v>0.026</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B4" s="14" t="n">
         <v>0</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1563,15 +1612,15 @@
         <v>1</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B6" s="10" t="n">
         <v>5</v>
@@ -1580,7 +1629,7 @@
         <v>35</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1617,118 +1666,118 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="21" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="5" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="E5" s="22" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F5" s="22" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1736,37 +1785,37 @@
     </row>
     <row r="11" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="F11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="F12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="F13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="F14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="F15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="F16" s="5"/>
     </row>

</xml_diff>